<commit_message>
Kleine Änderung an BM107 V6 BOM
Einzelpreis
</commit_message>
<xml_diff>
--- a/BM107/Labor_6_Schaltplan_Abgabe/BOM.xlsx
+++ b/BM107/Labor_6_Schaltplan_Abgabe/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\Documents\Uni\Semester 6\Projektarbeit\active-balancing\BM107\BM107_V6_Layout\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janne\Documents\GitHub\active-balancing\BM107\Labor_6_Schaltplan_Abgabe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{088CA72C-FBE2-4A52-940C-5AD3880A8D3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57DC1B69-B18E-46D2-8F8A-6DB633EC1B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4410" windowWidth="29040" windowHeight="15720" xr2:uid="{918699F1-1B84-4849-BAE5-2DB2563ABAC4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{918699F1-1B84-4849-BAE5-2DB2563ABAC4}"/>
   </bookViews>
   <sheets>
     <sheet name="BM107_V6_Layout" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="144">
   <si>
     <t>Reference</t>
   </si>
@@ -477,6 +477,12 @@
   </si>
   <si>
     <t>https://www.mouser.de/ProductDetail/Texas-Instruments/UCC27734QDRQ1?qs=PBDs2xEllI%2FilXPydpyARg%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">selber Preis </t>
+  </si>
+  <si>
+    <t>Stückpreis für eine Platine:</t>
   </si>
 </sst>
 </file>
@@ -487,7 +493,7 @@
     <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -505,6 +511,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -531,20 +545,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="20">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="12" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -611,25 +655,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3F77FE0A-A38E-4409-81C4-FAF5F65E10B1}" name="BM107_V6_Layout" displayName="BM107_V6_Layout" ref="A1:L40" tableType="queryTable" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3F77FE0A-A38E-4409-81C4-FAF5F65E10B1}" name="BM107_V6_Layout" displayName="BM107_V6_Layout" ref="A1:L41" tableType="queryTable" totalsRowCount="1">
   <autoFilter ref="A1:L40" xr:uid="{3F77FE0A-A38E-4409-81C4-FAF5F65E10B1}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{60E99FC0-45F6-4AB4-8FB6-D93C680A901A}" uniqueName="1" name="Reference" queryTableFieldId="1" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{60E99FC0-45F6-4AB4-8FB6-D93C680A901A}" uniqueName="1" name="Reference" queryTableFieldId="1" dataDxfId="19" totalsRowDxfId="8"/>
     <tableColumn id="2" xr3:uid="{3E3F015B-A0EE-458D-961C-068453D5CB7C}" uniqueName="2" name="Qty" queryTableFieldId="2"/>
-    <tableColumn id="3" xr3:uid="{9206E376-7C51-44EF-AECB-D096BE006700}" uniqueName="3" name="Value" queryTableFieldId="3" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{9B6378EC-E612-4806-AE3C-A4CE496C2ADD}" uniqueName="4" name="DNP" queryTableFieldId="4" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{F99D5491-8A41-4F46-8B8B-D8FB0E303CBD}" uniqueName="5" name="Exclude from BOM" queryTableFieldId="5" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{5C123A82-8310-482A-8170-0B1B8C78A17F}" uniqueName="6" name="Exclude from Board" queryTableFieldId="6" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{EE316574-29CC-4C34-BD36-9D6BF00A3113}" uniqueName="7" name="Footprint" queryTableFieldId="7" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{890D6B56-8EF6-4CA4-939B-C67156548BA1}" uniqueName="12" name="Stückzahl für 10 Platinen" queryTableFieldId="11" dataDxfId="4">
+    <tableColumn id="3" xr3:uid="{9206E376-7C51-44EF-AECB-D096BE006700}" uniqueName="3" name="Value" queryTableFieldId="3" dataDxfId="18" totalsRowDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{9B6378EC-E612-4806-AE3C-A4CE496C2ADD}" uniqueName="4" name="DNP" queryTableFieldId="4" dataDxfId="17" totalsRowDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{F99D5491-8A41-4F46-8B8B-D8FB0E303CBD}" uniqueName="5" name="Exclude from BOM" queryTableFieldId="5" dataDxfId="16" totalsRowDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{5C123A82-8310-482A-8170-0B1B8C78A17F}" uniqueName="6" name="Exclude from Board" queryTableFieldId="6" dataDxfId="15" totalsRowDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{EE316574-29CC-4C34-BD36-9D6BF00A3113}" uniqueName="7" name="Footprint" queryTableFieldId="7" dataDxfId="14" totalsRowDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{890D6B56-8EF6-4CA4-939B-C67156548BA1}" uniqueName="12" name="Stückzahl für 10 Platinen" queryTableFieldId="11" dataDxfId="13" totalsRowDxfId="2">
       <calculatedColumnFormula>BM107_V6_Layout[[#This Row],[Qty]]*10</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D0B85194-8D6F-4385-A736-061724C75029}" uniqueName="8" name="Kosten Stückzahl 10 (Preis pro 10 Stk*Stückzahl pro Platine)" queryTableFieldId="8" dataDxfId="3"/>
-    <tableColumn id="18" xr3:uid="{8EB1561F-2BE9-49AF-B44E-7407BEE40A17}" uniqueName="18" name="Stückzahl für 100 Platinen" queryTableFieldId="16" dataDxfId="2">
+    <tableColumn id="8" xr3:uid="{D0B85194-8D6F-4385-A736-061724C75029}" uniqueName="8" name="Kosten Stückzahl 10 (Preis pro 10 Stk*Stückzahl pro Platine)" queryTableFieldId="8" dataDxfId="12" totalsRowDxfId="1"/>
+    <tableColumn id="18" xr3:uid="{8EB1561F-2BE9-49AF-B44E-7407BEE40A17}" uniqueName="18" name="Stückzahl für 100 Platinen" queryTableFieldId="16" dataDxfId="11">
       <calculatedColumnFormula>BM107_V6_Layout[[#This Row],[Qty]]*100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{6F45B732-D151-4D43-B12D-A66A06D22536}" uniqueName="9" name="Kosten Stückzahl 100 (Preis pro 100 Stk*Stückzahl pro Platine)" queryTableFieldId="9" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{5A7D35DF-D8D2-4E89-B0FD-9A047A54CE32}" uniqueName="10" name="Quelle" queryTableFieldId="10" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{6F45B732-D151-4D43-B12D-A66A06D22536}" uniqueName="9" name="Kosten Stückzahl 100 (Preis pro 100 Stk*Stückzahl pro Platine)" queryTableFieldId="9" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{5A7D35DF-D8D2-4E89-B0FD-9A047A54CE32}" uniqueName="10" name="Quelle" queryTableFieldId="10" dataDxfId="10" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -952,24 +996,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE62859-B21F-43B8-B2EA-5034B1D08FF4}">
-  <dimension ref="A1:L40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L43"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="56.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.81640625" customWidth="1"/>
-    <col min="9" max="9" width="53.81640625" customWidth="1"/>
-    <col min="10" max="10" width="26.08984375" customWidth="1"/>
-    <col min="11" max="11" width="57.1796875" customWidth="1"/>
-    <col min="12" max="12" width="115.81640625" customWidth="1"/>
+    <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="56.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.77734375" customWidth="1"/>
+    <col min="9" max="9" width="53.77734375" customWidth="1"/>
+    <col min="10" max="10" width="26.109375" customWidth="1"/>
+    <col min="11" max="11" width="57.21875" customWidth="1"/>
+    <col min="12" max="12" width="115.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1007,7 +1051,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1049,7 +1093,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1091,7 +1135,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1133,7 +1177,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1175,7 +1219,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1217,7 +1261,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1259,7 +1303,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1301,7 +1345,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -1343,7 +1387,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1385,7 +1429,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -1427,7 +1471,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -1469,7 +1513,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -1511,7 +1555,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -1553,7 +1597,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>39</v>
       </c>
@@ -1595,7 +1639,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -1635,7 +1679,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>45</v>
       </c>
@@ -1675,7 +1719,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -1717,7 +1761,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1757,7 +1801,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -1797,7 +1841,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -1839,7 +1883,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -1879,7 +1923,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -1916,10 +1960,10 @@
         <v>1.93</v>
       </c>
       <c r="L23" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -1959,7 +2003,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>67</v>
       </c>
@@ -2001,7 +2045,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>69</v>
       </c>
@@ -2043,7 +2087,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>71</v>
       </c>
@@ -2083,7 +2127,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>73</v>
       </c>
@@ -2123,7 +2167,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>75</v>
       </c>
@@ -2163,7 +2207,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>77</v>
       </c>
@@ -2203,7 +2247,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>79</v>
       </c>
@@ -2243,7 +2287,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>82</v>
       </c>
@@ -2283,7 +2327,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>85</v>
       </c>
@@ -2323,7 +2367,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>88</v>
       </c>
@@ -2363,7 +2407,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>91</v>
       </c>
@@ -2403,7 +2447,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>93</v>
       </c>
@@ -2443,7 +2487,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>96</v>
       </c>
@@ -2483,7 +2527,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>98</v>
       </c>
@@ -2523,7 +2567,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>101</v>
       </c>
@@ -2563,7 +2607,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>103</v>
       </c>
@@ -2601,6 +2645,35 @@
       </c>
       <c r="L40" t="s">
         <v>141</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="L41" s="5"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="I42" t="s">
+        <v>143</v>
+      </c>
+      <c r="K42" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="I43" s="7">
+        <f>SUM(I5:I40)/10</f>
+        <v>80.337999999999994</v>
+      </c>
+      <c r="K43" s="6">
+        <f>SUM(K5:K40)/100</f>
+        <v>61.352235999999991</v>
       </c>
     </row>
   </sheetData>
@@ -2620,7 +2693,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CFAE9DB-21E6-4B31-BFCB-8BDB277A0622}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>